<commit_message>
Small updates and added some data files
</commit_message>
<xml_diff>
--- a/data/carbon_factors.xlsx
+++ b/data/carbon_factors.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/corra_joseph_epa_gov/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/corra_joseph_epa_gov/Documents/Profile/Documents/Fossil Fuels/Fossil Fuels/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{272D798C-3231-4784-9687-9176A8284688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{339D6A27-6B34-4218-8715-C3F9D34524D3}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="8_{272D798C-3231-4784-9687-9176A8284688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{57C7A81F-3ACB-40FB-B957-61B417136D85}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{3ECB161D-927E-4A86-B5AC-7932B52A7390}"/>
+    <workbookView xWindow="34530" yWindow="3540" windowWidth="19680" windowHeight="10635" activeTab="1" xr2:uid="{3ECB161D-927E-4A86-B5AC-7932B52A7390}"/>
   </bookViews>
   <sheets>
     <sheet name="factors_variable" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="64">
   <si>
     <t>Fuel Type</t>
   </si>
@@ -108,9 +108,6 @@
     <t>NC</t>
   </si>
   <si>
-    <t>Electric Utility Coal</t>
-  </si>
-  <si>
     <t>U.S. Territory Coal Imports (Bit.)</t>
   </si>
   <si>
@@ -138,9 +135,6 @@
     <t>Aviation Gasoline</t>
   </si>
   <si>
-    <t>Jet Fuel (Kerosene)</t>
-  </si>
-  <si>
     <t>Kerosene</t>
   </si>
   <si>
@@ -220,6 +214,21 @@
   </si>
   <si>
     <t>Motor Gasoline (Light-Duty Vehicles)</t>
+  </si>
+  <si>
+    <t>fraction_oxidized</t>
+  </si>
+  <si>
+    <t>fraction_neu_sequestered</t>
+  </si>
+  <si>
+    <t>carbon_coefficient</t>
+  </si>
+  <si>
+    <t>heat_content</t>
+  </si>
+  <si>
+    <t>fuel_type</t>
   </si>
 </sst>
 </file>
@@ -2352,34 +2361,42 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42871F84-221D-4A86-8B12-0CC25BD2B03B}">
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="3" width="18" customWidth="1"/>
+    <col min="4" max="5" width="10.7265625" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>17</v>
+        <v>63</v>
       </c>
       <c r="B1" t="s">
-        <v>18</v>
+        <v>62</v>
+      </c>
+      <c r="C1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E1" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" t="s">
         <v>19</v>
@@ -2393,7 +2410,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="B4" t="s">
         <v>19</v>
@@ -2403,14 +2420,11 @@
       </c>
       <c r="D4">
         <v>1</v>
-      </c>
-      <c r="E4">
-        <v>0.1</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="B5" t="s">
         <v>19</v>
@@ -2420,17 +2434,20 @@
       </c>
       <c r="D5">
         <v>1</v>
+      </c>
+      <c r="E5">
+        <v>0.1</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="B6" t="s">
         <v>19</v>
       </c>
-      <c r="C6">
-        <v>27.85</v>
+      <c r="C6" t="s">
+        <v>19</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -2438,41 +2455,41 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>22</v>
-      </c>
-      <c r="C7" t="s">
-        <v>22</v>
-      </c>
-      <c r="D7" t="s">
-        <v>22</v>
+        <v>19</v>
+      </c>
+      <c r="C7">
+        <v>27.85</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D8">
-        <v>1</v>
+        <v>22</v>
+      </c>
+      <c r="D8" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>24</v>
-      </c>
-      <c r="B9">
-        <v>22.3</v>
-      </c>
-      <c r="C9">
-        <v>25.14</v>
+        <v>4</v>
+      </c>
+      <c r="B9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" t="s">
+        <v>19</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -2480,10 +2497,16 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" t="s">
-        <v>25</v>
+        <v>23</v>
+      </c>
+      <c r="B10">
+        <v>22.3</v>
+      </c>
+      <c r="C10">
+        <v>25.14</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
@@ -2491,127 +2514,121 @@
         <v>14</v>
       </c>
       <c r="B11" t="s">
-        <v>19</v>
-      </c>
-      <c r="C11" t="s">
-        <v>19</v>
-      </c>
-      <c r="D11">
-        <v>1</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>26</v>
-      </c>
-      <c r="C12">
-        <v>14.47</v>
-      </c>
-      <c r="E12">
-        <v>0</v>
+        <v>14</v>
+      </c>
+      <c r="B12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C13">
         <v>14.47</v>
       </c>
-      <c r="E13" t="s">
-        <v>19</v>
+      <c r="E13">
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C14">
-        <v>14.92</v>
-      </c>
-      <c r="D14">
-        <v>1</v>
+        <v>14.47</v>
+      </c>
+      <c r="E14" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>29</v>
-      </c>
-      <c r="B15" t="s">
-        <v>30</v>
+        <v>27</v>
+      </c>
+      <c r="C15">
+        <v>14.92</v>
+      </c>
+      <c r="D15">
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>31</v>
-      </c>
-      <c r="B16">
-        <v>6.6360000000000001</v>
-      </c>
-      <c r="C16">
-        <v>20.55318099621897</v>
-      </c>
-      <c r="D16">
-        <v>1</v>
-      </c>
-      <c r="E16">
-        <v>0.99560852232832731</v>
+        <v>28</v>
+      </c>
+      <c r="B16" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B17">
-        <v>5.048</v>
+        <v>6.6360000000000001</v>
       </c>
       <c r="C17">
-        <v>18.855352254718337</v>
+        <v>20.55318099621897</v>
       </c>
       <c r="D17">
         <v>1</v>
+      </c>
+      <c r="E17">
+        <v>0.99560852232832731</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>15</v>
-      </c>
-      <c r="B18" t="s">
-        <v>19</v>
-      </c>
-      <c r="C18" t="s">
-        <v>19</v>
+        <v>31</v>
+      </c>
+      <c r="B18">
+        <v>5.048</v>
+      </c>
+      <c r="C18">
+        <v>18.855352254718337</v>
       </c>
       <c r="D18">
         <v>1</v>
-      </c>
-      <c r="E18">
-        <v>0.5</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>33</v>
-      </c>
-      <c r="B19">
-        <v>5.67</v>
+        <v>15</v>
+      </c>
+      <c r="B19" t="s">
+        <v>19</v>
       </c>
       <c r="C19" t="s">
         <v>19</v>
       </c>
       <c r="D19">
         <v>1</v>
+      </c>
+      <c r="E19">
+        <v>0.5</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="B20">
         <v>5.67</v>
       </c>
-      <c r="C20">
-        <v>19.964104564962931</v>
+      <c r="C20" t="s">
+        <v>19</v>
       </c>
       <c r="D20">
         <v>1</v>
@@ -2619,13 +2636,13 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B21">
         <v>5.67</v>
       </c>
       <c r="C21">
-        <v>19.329999999999998</v>
+        <v>19.964104564962931</v>
       </c>
       <c r="D21">
         <v>1</v>
@@ -2633,13 +2650,13 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="B22">
-        <v>3.8410000000000002</v>
-      </c>
-      <c r="C22" t="s">
-        <v>19</v>
+        <v>5.67</v>
+      </c>
+      <c r="C22">
+        <v>19.329999999999998</v>
       </c>
       <c r="D22">
         <v>1</v>
@@ -2647,10 +2664,10 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>36</v>
+        <v>5</v>
       </c>
       <c r="B23">
-        <v>3.867</v>
+        <v>3.8410000000000002</v>
       </c>
       <c r="C23" t="s">
         <v>19</v>
@@ -2661,58 +2678,58 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>37</v>
-      </c>
-      <c r="B24" t="s">
-        <v>19</v>
+        <v>34</v>
+      </c>
+      <c r="B24">
+        <v>3.867</v>
       </c>
       <c r="C24" t="s">
         <v>19</v>
       </c>
-      <c r="E24" t="s">
-        <v>19</v>
+      <c r="D24">
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>38</v>
-      </c>
-      <c r="B25">
-        <v>6.0650000000000004</v>
-      </c>
-      <c r="C25">
-        <v>20.199355467286214</v>
-      </c>
-      <c r="D25">
-        <v>1</v>
-      </c>
-      <c r="E25">
-        <v>9.1799999999999993E-2</v>
+        <v>35</v>
+      </c>
+      <c r="B25" t="s">
+        <v>19</v>
+      </c>
+      <c r="C25" t="s">
+        <v>19</v>
+      </c>
+      <c r="E25" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>8</v>
-      </c>
-      <c r="B26" t="s">
-        <v>19</v>
-      </c>
-      <c r="C26" t="s">
-        <v>19</v>
+        <v>36</v>
+      </c>
+      <c r="B26">
+        <v>6.0650000000000004</v>
+      </c>
+      <c r="C26">
+        <v>20.199355467286214</v>
       </c>
       <c r="D26">
         <v>1</v>
+      </c>
+      <c r="E26">
+        <v>9.1799999999999993E-2</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>39</v>
+        <v>8</v>
       </c>
       <c r="B27" t="s">
         <v>19</v>
       </c>
-      <c r="C27">
-        <v>19.22</v>
+      <c r="C27" t="s">
+        <v>19</v>
       </c>
       <c r="D27">
         <v>1</v>
@@ -2720,63 +2737,63 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>40</v>
-      </c>
-      <c r="B28">
-        <v>6.2869999999999999</v>
+        <v>37</v>
+      </c>
+      <c r="B28" t="s">
+        <v>19</v>
       </c>
       <c r="C28">
-        <v>20.48</v>
+        <v>19.22</v>
       </c>
       <c r="D28">
         <v>1</v>
-      </c>
-      <c r="E28">
-        <v>0.5</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B29">
-        <v>5.2480000000000002</v>
+        <v>6.2869999999999999</v>
       </c>
       <c r="C29">
-        <v>19.737389135254986</v>
+        <v>20.48</v>
       </c>
       <c r="D29">
         <v>1</v>
       </c>
-      <c r="E29" t="s">
-        <v>19</v>
+      <c r="E29">
+        <v>0.5</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>42</v>
+        <v>39</v>
+      </c>
+      <c r="B30">
+        <v>5.2480000000000002</v>
+      </c>
+      <c r="C30">
+        <v>19.737389135254986</v>
+      </c>
+      <c r="D30">
+        <v>1</v>
+      </c>
+      <c r="E30" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>43</v>
-      </c>
-      <c r="C31">
-        <v>18.87</v>
-      </c>
-      <c r="D31">
-        <v>1</v>
+        <v>40</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>13</v>
-      </c>
-      <c r="B32">
-        <v>5.8</v>
-      </c>
-      <c r="C32" t="s">
-        <v>19</v>
+        <v>41</v>
+      </c>
+      <c r="C32">
+        <v>18.87</v>
       </c>
       <c r="D32">
         <v>1</v>
@@ -2784,7 +2801,10 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>10</v>
+        <v>13</v>
+      </c>
+      <c r="B33">
+        <v>5.8</v>
       </c>
       <c r="C33" t="s">
         <v>19</v>
@@ -2795,64 +2815,58 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>11</v>
-      </c>
-      <c r="B34">
-        <v>5.7960000000000003</v>
+        <v>10</v>
       </c>
       <c r="C34" t="s">
         <v>19</v>
       </c>
       <c r="D34">
         <v>1</v>
-      </c>
-      <c r="E34">
-        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>44</v>
+        <v>11</v>
       </c>
       <c r="B35">
-        <v>5.8</v>
-      </c>
-      <c r="C35">
-        <v>20</v>
+        <v>5.7960000000000003</v>
+      </c>
+      <c r="C35" t="s">
+        <v>19</v>
       </c>
       <c r="D35">
         <v>1</v>
       </c>
       <c r="E35">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B36">
-        <v>5.2480000000000002</v>
+        <v>5.8</v>
       </c>
       <c r="C36">
-        <v>18.550649350649344</v>
+        <v>20</v>
       </c>
       <c r="D36">
         <v>1</v>
       </c>
-      <c r="E36" t="s">
-        <v>19</v>
+      <c r="E36">
+        <v>0.1</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B37">
-        <v>5.8250000000000002</v>
+        <v>5.2480000000000002</v>
       </c>
       <c r="C37">
-        <v>20.170000000000002</v>
+        <v>18.550649350649344</v>
       </c>
       <c r="D37">
         <v>1</v>
@@ -2863,13 +2877,13 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B38">
-        <v>4.6379999999999999</v>
+        <v>5.8250000000000002</v>
       </c>
       <c r="C38">
-        <v>18.239999999999998</v>
+        <v>20.170000000000002</v>
       </c>
       <c r="D38">
         <v>1</v>
@@ -2880,13 +2894,13 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>48</v>
-      </c>
-      <c r="B39" t="s">
-        <v>49</v>
+        <v>45</v>
+      </c>
+      <c r="B39">
+        <v>4.6379999999999999</v>
       </c>
       <c r="C39">
-        <v>19.37</v>
+        <v>18.239999999999998</v>
       </c>
       <c r="D39">
         <v>1</v>
@@ -2897,44 +2911,47 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>50</v>
-      </c>
-      <c r="B40">
-        <v>6.024</v>
+        <v>46</v>
+      </c>
+      <c r="B40" t="s">
+        <v>47</v>
       </c>
       <c r="C40">
-        <v>27.84770010865628</v>
+        <v>19.37</v>
       </c>
       <c r="D40">
         <v>1</v>
       </c>
-      <c r="E40">
-        <v>0.3</v>
+      <c r="E40" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B41">
-        <v>4.62</v>
+        <v>6.024</v>
       </c>
       <c r="C41">
-        <v>18.239999999999998</v>
+        <v>27.84770010865628</v>
       </c>
       <c r="D41">
         <v>1</v>
+      </c>
+      <c r="E41">
+        <v>0.3</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B42">
-        <v>5.4180000000000001</v>
+        <v>4.62</v>
       </c>
       <c r="C42">
-        <v>19.41</v>
+        <v>18.239999999999998</v>
       </c>
       <c r="D42">
         <v>1</v>
@@ -2942,13 +2959,13 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B43">
-        <v>6</v>
+        <v>5.4180000000000001</v>
       </c>
       <c r="C43">
-        <v>18.195454545454545</v>
+        <v>19.41</v>
       </c>
       <c r="D43">
         <v>1</v>
@@ -2956,44 +2973,44 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B44">
         <v>6</v>
       </c>
       <c r="C44">
-        <v>17.510000000000002</v>
-      </c>
-      <c r="D44" t="s">
-        <v>55</v>
-      </c>
-      <c r="E44" t="s">
-        <v>19</v>
+        <v>18.195454545454545</v>
+      </c>
+      <c r="D44">
+        <v>1</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>12</v>
+        <v>52</v>
       </c>
       <c r="B45">
-        <v>5.8250000000000002</v>
-      </c>
-      <c r="C45" t="s">
-        <v>19</v>
-      </c>
-      <c r="D45">
-        <v>1</v>
+        <v>6</v>
+      </c>
+      <c r="C45">
+        <v>17.510000000000002</v>
+      </c>
+      <c r="D45" t="s">
+        <v>53</v>
+      </c>
+      <c r="E45" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>56</v>
+        <v>12</v>
       </c>
       <c r="B46">
-        <v>5.4180000000000001</v>
-      </c>
-      <c r="C46">
-        <v>19.41</v>
+        <v>5.8250000000000002</v>
+      </c>
+      <c r="C46" t="s">
+        <v>19</v>
       </c>
       <c r="D46">
         <v>1</v>
@@ -3001,54 +3018,68 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B47">
-        <v>5.5369999999999999</v>
+        <v>5.4180000000000001</v>
       </c>
       <c r="C47">
-        <v>19.795754182606267</v>
+        <v>19.41</v>
       </c>
       <c r="D47">
         <v>1</v>
-      </c>
-      <c r="E47">
-        <v>0.57824999999999982</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>58</v>
+        <v>55</v>
+      </c>
+      <c r="B48">
+        <v>5.5369999999999999</v>
       </c>
       <c r="C48">
-        <v>2.6974658424810825</v>
+        <v>19.795754182606267</v>
       </c>
       <c r="D48">
         <v>1</v>
+      </c>
+      <c r="E48">
+        <v>0.57824999999999982</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>59</v>
-      </c>
-      <c r="B49">
-        <v>6.2869999999999999</v>
+        <v>56</v>
       </c>
       <c r="C49">
-        <v>21.29</v>
+        <v>2.6974658424810825</v>
       </c>
       <c r="D49">
         <v>1</v>
-      </c>
-      <c r="E49">
-        <v>0.5</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>60</v>
+        <v>57</v>
+      </c>
+      <c r="B50">
+        <v>6.2869999999999999</v>
+      </c>
+      <c r="C50">
+        <v>21.29</v>
       </c>
       <c r="D50">
+        <v>1</v>
+      </c>
+      <c r="E50">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>58</v>
+      </c>
+      <c r="D51">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fixed some issues with SEDS (repeated unit conversions).Commented out some code that is not currently being used (2025).
</commit_message>
<xml_diff>
--- a/data/carbon_factors.xlsx
+++ b/data/carbon_factors.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/corra_joseph_epa_gov/Documents/Profile/Documents/Fossil Fuels/Fossil Fuels/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="8_{272D798C-3231-4784-9687-9176A8284688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{57C7A81F-3ACB-40FB-B957-61B417136D85}"/>
+  <xr:revisionPtr revIDLastSave="46" documentId="8_{272D798C-3231-4784-9687-9176A8284688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E780C507-C4C9-4F29-AFF8-88E705F1B8D5}"/>
   <bookViews>
-    <workbookView xWindow="34530" yWindow="3540" windowWidth="19680" windowHeight="10635" activeTab="1" xr2:uid="{3ECB161D-927E-4A86-B5AC-7932B52A7390}"/>
+    <workbookView xWindow="28680" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{3ECB161D-927E-4A86-B5AC-7932B52A7390}"/>
   </bookViews>
   <sheets>
     <sheet name="factors_variable" sheetId="1" r:id="rId1"/>
@@ -580,13 +580,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04583640-4A08-41EF-9B43-988CA299CA6B}">
-  <dimension ref="A1:AH17"/>
+  <dimension ref="A1:AI17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -689,8 +689,11 @@
       <c r="AH1">
         <v>2022</v>
       </c>
-    </row>
-    <row r="2" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="AI1">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -793,8 +796,11 @@
       <c r="AH2">
         <v>26.17943592337086</v>
       </c>
-    </row>
-    <row r="3" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="AI2">
+        <v>26.376336866994436</v>
+      </c>
+    </row>
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -897,8 +903,11 @@
       <c r="AH3">
         <v>26.17943592337086</v>
       </c>
-    </row>
-    <row r="4" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="AI3">
+        <v>26.376336866994436</v>
+      </c>
+    </row>
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1001,8 +1010,11 @@
       <c r="AH4">
         <v>26.104948569451711</v>
       </c>
-    </row>
-    <row r="5" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="AI4">
+        <v>26.121261544871881</v>
+      </c>
+    </row>
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -1105,8 +1117,11 @@
       <c r="AH5">
         <v>26.134701137600572</v>
       </c>
-    </row>
-    <row r="6" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="AI5">
+        <v>26.150731599716178</v>
+      </c>
+    </row>
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -1209,8 +1224,11 @@
       <c r="AH6">
         <v>17.146363636363635</v>
       </c>
-    </row>
-    <row r="7" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="AI6">
+        <v>17.146363636363635</v>
+      </c>
+    </row>
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -1313,8 +1331,11 @@
       <c r="AH7">
         <v>17.757127425341324</v>
       </c>
-    </row>
-    <row r="8" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="AI7">
+        <v>17.767768511281655</v>
+      </c>
+    </row>
+    <row r="8" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -1418,7 +1439,7 @@
         <v>16.816422899006234</v>
       </c>
     </row>
-    <row r="9" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -1521,8 +1542,11 @@
       <c r="AH9">
         <v>19.26959818755628</v>
       </c>
-    </row>
-    <row r="10" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="AI9">
+        <v>19.26959818755628</v>
+      </c>
+    </row>
+    <row r="10" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -1625,8 +1649,11 @@
       <c r="AH10">
         <v>19.696969696969692</v>
       </c>
-    </row>
-    <row r="11" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="AI10">
+        <v>19.696969696969692</v>
+      </c>
+    </row>
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -1729,8 +1756,11 @@
       <c r="AH11">
         <v>19.456118437849259</v>
       </c>
-    </row>
-    <row r="12" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="AI11">
+        <v>19.456118437849259</v>
+      </c>
+    </row>
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -1833,8 +1863,11 @@
       <c r="AH12">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="AI12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -1937,8 +1970,11 @@
       <c r="AH13">
         <v>20.305515594827586</v>
       </c>
-    </row>
-    <row r="14" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="AI13">
+        <v>20.305515594827586</v>
+      </c>
+    </row>
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -2041,8 +2077,11 @@
       <c r="AH14">
         <v>20.305515594827586</v>
       </c>
-    </row>
-    <row r="15" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="AI14">
+        <v>20.305515594827586</v>
+      </c>
+    </row>
+    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -2145,8 +2184,11 @@
       <c r="AH15">
         <v>14.431959663127413</v>
       </c>
-    </row>
-    <row r="16" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="AI15">
+        <v>14.431959663127413</v>
+      </c>
+    </row>
+    <row r="16" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>15</v>
       </c>
@@ -2249,8 +2291,11 @@
       <c r="AH16">
         <v>20.216892495282984</v>
       </c>
-    </row>
-    <row r="17" spans="1:34" x14ac:dyDescent="0.35">
+      <c r="AI16">
+        <v>20.216892495282984</v>
+      </c>
+    </row>
+    <row r="17" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -2353,9 +2398,13 @@
       <c r="AH17">
         <v>25.605077665523787</v>
       </c>
+      <c r="AI17">
+        <v>25.605077665523801</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Updated to accommodate 2025 state inventory. contains some temporary slapdash code to expedite state Inventory compilation (i.e., circumvents national emissions compilation)
</commit_message>
<xml_diff>
--- a/data/carbon_factors.xlsx
+++ b/data/carbon_factors.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/corra_joseph_epa_gov/Documents/Profile/Documents/Fossil Fuels/Fossil Fuels/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="46" documentId="8_{272D798C-3231-4784-9687-9176A8284688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E780C507-C4C9-4F29-AFF8-88E705F1B8D5}"/>
+  <xr:revisionPtr revIDLastSave="50" documentId="8_{272D798C-3231-4784-9687-9176A8284688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{35C88EEE-5260-4D6E-9AB0-FD150A107D82}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{3ECB161D-927E-4A86-B5AC-7932B52A7390}"/>
+    <workbookView xWindow="28680" yWindow="-60" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{3ECB161D-927E-4A86-B5AC-7932B52A7390}"/>
   </bookViews>
   <sheets>
     <sheet name="factors_variable" sheetId="1" r:id="rId1"/>
@@ -54,9 +54,6 @@
     <t>Electric Power Coal</t>
   </si>
   <si>
-    <t>LPG (Propane)</t>
-  </si>
-  <si>
     <t>HGL (Energy Use)</t>
   </si>
   <si>
@@ -153,9 +150,6 @@
     <t>Motor Gasoline (Territories)</t>
   </si>
   <si>
-    <t>Residual Fuel</t>
-  </si>
-  <si>
     <t>Special Naphtha</t>
   </si>
   <si>
@@ -207,9 +201,6 @@
     <t>Waxes</t>
   </si>
   <si>
-    <t>Geothermal</t>
-  </si>
-  <si>
     <t>Special Factor for Utility Sector Residual Fuel</t>
   </si>
   <si>
@@ -229,6 +220,15 @@
   </si>
   <si>
     <t>fuel_type</t>
+  </si>
+  <si>
+    <t>LPG</t>
+  </si>
+  <si>
+    <t>Residual Fuel Oil</t>
+  </si>
+  <si>
+    <t>Geothermal Energy</t>
   </si>
 </sst>
 </file>
@@ -1123,7 +1123,7 @@
     </row>
     <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>5</v>
+        <v>61</v>
       </c>
       <c r="B6">
         <v>17.146363636363635</v>
@@ -1230,7 +1230,7 @@
     </row>
     <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B7">
         <v>17.401801615264294</v>
@@ -1337,7 +1337,7 @@
     </row>
     <row r="8" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8">
         <v>17.206134812379201</v>
@@ -1441,7 +1441,7 @@
     </row>
     <row r="9" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B9">
         <v>19.422820377744564</v>
@@ -1548,7 +1548,7 @@
     </row>
     <row r="10" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B10">
         <v>19.399999999999999</v>
@@ -1655,7 +1655,7 @@
     </row>
     <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11">
         <v>19.422820377744564</v>
@@ -1762,7 +1762,7 @@
     </row>
     <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -1869,7 +1869,7 @@
     </row>
     <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13">
         <v>20.14625771551724</v>
@@ -1976,7 +1976,7 @@
     </row>
     <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B14">
         <v>20.14625771551724</v>
@@ -2083,7 +2083,7 @@
     </row>
     <row r="15" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B15">
         <v>14.455165742468415</v>
@@ -2190,7 +2190,7 @@
     </row>
     <row r="16" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B16">
         <v>20.170000000000002</v>
@@ -2297,7 +2297,7 @@
     </row>
     <row r="17" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B17">
         <v>25.532291814167994</v>
@@ -2420,27 +2420,27 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C1" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D1" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" t="s">
         <v>17</v>
-      </c>
-      <c r="B2" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -2448,10 +2448,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -2462,10 +2462,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -2473,13 +2473,13 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -2493,10 +2493,10 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -2504,10 +2504,10 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C7">
         <v>27.85</v>
@@ -2518,16 +2518,16 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" t="s">
         <v>21</v>
       </c>
-      <c r="B8" t="s">
-        <v>22</v>
-      </c>
       <c r="C8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
@@ -2535,10 +2535,10 @@
         <v>4</v>
       </c>
       <c r="B9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -2546,7 +2546,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B10">
         <v>22.3</v>
@@ -2560,21 +2560,21 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C12" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -2582,7 +2582,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C13">
         <v>14.47</v>
@@ -2593,18 +2593,18 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C14">
         <v>14.47</v>
       </c>
       <c r="E14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C15">
         <v>14.92</v>
@@ -2615,15 +2615,15 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" t="s">
         <v>28</v>
-      </c>
-      <c r="B16" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B17">
         <v>6.6360000000000001</v>
@@ -2640,7 +2640,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B18">
         <v>5.048</v>
@@ -2654,13 +2654,13 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B19" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C19" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D19">
         <v>1</v>
@@ -2671,13 +2671,13 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B20">
         <v>5.67</v>
       </c>
       <c r="C20" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D20">
         <v>1</v>
@@ -2685,7 +2685,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B21">
         <v>5.67</v>
@@ -2699,7 +2699,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B22">
         <v>5.67</v>
@@ -2713,13 +2713,13 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>5</v>
+        <v>61</v>
       </c>
       <c r="B23">
         <v>3.8410000000000002</v>
       </c>
       <c r="C23" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D23">
         <v>1</v>
@@ -2727,13 +2727,13 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B24">
         <v>3.867</v>
       </c>
       <c r="C24" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D24">
         <v>1</v>
@@ -2741,21 +2741,21 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B25" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C25" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E25" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B26">
         <v>6.0650000000000004</v>
@@ -2772,13 +2772,13 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B27" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C27" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D27">
         <v>1</v>
@@ -2786,10 +2786,10 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B28" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C28">
         <v>19.22</v>
@@ -2800,7 +2800,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>38</v>
+        <v>62</v>
       </c>
       <c r="B29">
         <v>6.2869999999999999</v>
@@ -2817,7 +2817,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B30">
         <v>5.2480000000000002</v>
@@ -2829,17 +2829,17 @@
         <v>1</v>
       </c>
       <c r="E30" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C32">
         <v>18.87</v>
@@ -2850,13 +2850,13 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B33">
         <v>5.8</v>
       </c>
       <c r="C33" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D33">
         <v>1</v>
@@ -2864,10 +2864,10 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C34" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D34">
         <v>1</v>
@@ -2875,13 +2875,13 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B35">
         <v>5.7960000000000003</v>
       </c>
       <c r="C35" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D35">
         <v>1</v>
@@ -2892,7 +2892,7 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B36">
         <v>5.8</v>
@@ -2909,7 +2909,7 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B37">
         <v>5.2480000000000002</v>
@@ -2921,12 +2921,12 @@
         <v>1</v>
       </c>
       <c r="E37" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B38">
         <v>5.8250000000000002</v>
@@ -2938,12 +2938,12 @@
         <v>1</v>
       </c>
       <c r="E38" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B39">
         <v>4.6379999999999999</v>
@@ -2955,15 +2955,15 @@
         <v>1</v>
       </c>
       <c r="E39" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B40" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C40">
         <v>19.37</v>
@@ -2972,12 +2972,12 @@
         <v>1</v>
       </c>
       <c r="E40" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B41">
         <v>6.024</v>
@@ -2994,7 +2994,7 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B42">
         <v>4.62</v>
@@ -3008,7 +3008,7 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B43">
         <v>5.4180000000000001</v>
@@ -3022,7 +3022,7 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B44">
         <v>6</v>
@@ -3036,7 +3036,7 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B45">
         <v>6</v>
@@ -3045,21 +3045,21 @@
         <v>17.510000000000002</v>
       </c>
       <c r="D45" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E45" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B46">
         <v>5.8250000000000002</v>
       </c>
       <c r="C46" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D46">
         <v>1</v>
@@ -3067,7 +3067,7 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B47">
         <v>5.4180000000000001</v>
@@ -3081,7 +3081,7 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B48">
         <v>5.5369999999999999</v>
@@ -3098,7 +3098,7 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="C49">
         <v>2.6974658424810825</v>
@@ -3109,7 +3109,7 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B50">
         <v>6.2869999999999999</v>
@@ -3126,7 +3126,7 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D51">
         <v>1</v>

</xml_diff>

<commit_message>
Continued work trying to make final values match previous years
</commit_message>
<xml_diff>
--- a/data/carbon_factors.xlsx
+++ b/data/carbon_factors.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/corra_joseph_epa_gov/Documents/Profile/Documents/Fossil Fuels/Fossil Fuels/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="50" documentId="8_{272D798C-3231-4784-9687-9176A8284688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{35C88EEE-5260-4D6E-9AB0-FD150A107D82}"/>
+  <xr:revisionPtr revIDLastSave="57" documentId="8_{272D798C-3231-4784-9687-9176A8284688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2F76F547-F673-4F6F-82D5-3147B591BADA}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-60" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{3ECB161D-927E-4A86-B5AC-7932B52A7390}"/>
   </bookViews>
@@ -162,12 +162,6 @@
     <t>Misc. Products (Territories)</t>
   </si>
   <si>
-    <t>Naphtha (&lt;401 deg. F)</t>
-  </si>
-  <si>
-    <t>Other Oil (&gt;401 deg. F)</t>
-  </si>
-  <si>
     <t>Pentanes Plus</t>
   </si>
   <si>
@@ -229,6 +223,12 @@
   </si>
   <si>
     <t>Geothermal Energy</t>
+  </si>
+  <si>
+    <t>Naphtha</t>
+  </si>
+  <si>
+    <t>Other Oils</t>
   </si>
 </sst>
 </file>
@@ -1123,7 +1123,7 @@
     </row>
     <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B6">
         <v>17.146363636363635</v>
@@ -1438,6 +1438,9 @@
       <c r="AH8">
         <v>16.816422899006234</v>
       </c>
+      <c r="AI8">
+        <v>16.805926972403768</v>
+      </c>
     </row>
     <row r="9" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
@@ -2399,7 +2402,7 @@
         <v>25.605077665523787</v>
       </c>
       <c r="AI17">
-        <v>25.605077665523801</v>
+        <v>25.594268546685665</v>
       </c>
     </row>
   </sheetData>
@@ -2420,19 +2423,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
@@ -2713,7 +2716,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B23">
         <v>3.8410000000000002</v>
@@ -2800,7 +2803,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B29">
         <v>6.2869999999999999</v>
@@ -2909,7 +2912,7 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>41</v>
+        <v>62</v>
       </c>
       <c r="B37">
         <v>5.2480000000000002</v>
@@ -2926,7 +2929,7 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="B38">
         <v>5.8250000000000002</v>
@@ -2943,7 +2946,7 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B39">
         <v>4.6379999999999999</v>
@@ -2960,10 +2963,10 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B40" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C40">
         <v>19.37</v>
@@ -2977,7 +2980,7 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B41">
         <v>6.024</v>
@@ -2994,7 +2997,7 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B42">
         <v>4.62</v>
@@ -3008,7 +3011,7 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B43">
         <v>5.4180000000000001</v>
@@ -3022,7 +3025,7 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B44">
         <v>6</v>
@@ -3036,7 +3039,7 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B45">
         <v>6</v>
@@ -3045,7 +3048,7 @@
         <v>17.510000000000002</v>
       </c>
       <c r="D45" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E45" t="s">
         <v>18</v>
@@ -3067,7 +3070,7 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B47">
         <v>5.4180000000000001</v>
@@ -3081,7 +3084,7 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B48">
         <v>5.5369999999999999</v>
@@ -3098,7 +3101,7 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C49">
         <v>2.6974658424810825</v>
@@ -3109,7 +3112,7 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B50">
         <v>6.2869999999999999</v>
@@ -3126,7 +3129,7 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D51">
         <v>1</v>

</xml_diff>

<commit_message>
Lots of little changes to fix minor errors in state calculations. Will need to be reorganized at some point.
Also edited raw data due to annoying naming discrepancies.
</commit_message>
<xml_diff>
--- a/data/carbon_factors.xlsx
+++ b/data/carbon_factors.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/corra_joseph_epa_gov/Documents/Profile/Documents/Fossil Fuels/Fossil Fuels/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="57" documentId="8_{272D798C-3231-4784-9687-9176A8284688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2F76F547-F673-4F6F-82D5-3147B591BADA}"/>
+  <xr:revisionPtr revIDLastSave="59" documentId="8_{272D798C-3231-4784-9687-9176A8284688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4509351-B9C7-4A45-A634-A90D0519E190}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-60" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{3ECB161D-927E-4A86-B5AC-7932B52A7390}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="63">
   <si>
     <t>Fuel Type</t>
   </si>
@@ -136,9 +136,6 @@
   </si>
   <si>
     <t>Jet Fuel &amp; Kerosene (Territories)</t>
-  </si>
-  <si>
-    <t>HGL (energy use/Territories)</t>
   </si>
   <si>
     <t>HGL (non-energy use)</t>
@@ -1123,7 +1120,7 @@
     </row>
     <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B6">
         <v>17.146363636363635</v>
@@ -2423,19 +2420,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1" t="s">
         <v>54</v>
-      </c>
-      <c r="E1" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
@@ -2716,7 +2713,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B23">
         <v>3.8410000000000002</v>
@@ -2730,7 +2727,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="B24">
         <v>3.867</v>
@@ -2744,7 +2741,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B25" t="s">
         <v>18</v>
@@ -2758,7 +2755,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B26">
         <v>6.0650000000000004</v>
@@ -2789,7 +2786,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B28" t="s">
         <v>18</v>
@@ -2803,7 +2800,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B29">
         <v>6.2869999999999999</v>
@@ -2820,7 +2817,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B30">
         <v>5.2480000000000002</v>
@@ -2837,12 +2834,12 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C32">
         <v>18.87</v>
@@ -2895,7 +2892,7 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B36">
         <v>5.8</v>
@@ -2912,7 +2909,7 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B37">
         <v>5.2480000000000002</v>
@@ -2929,7 +2926,7 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B38">
         <v>5.8250000000000002</v>
@@ -2946,7 +2943,7 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B39">
         <v>4.6379999999999999</v>
@@ -2963,10 +2960,10 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
+        <v>41</v>
+      </c>
+      <c r="B40" t="s">
         <v>42</v>
-      </c>
-      <c r="B40" t="s">
-        <v>43</v>
       </c>
       <c r="C40">
         <v>19.37</v>
@@ -2980,7 +2977,7 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B41">
         <v>6.024</v>
@@ -2997,7 +2994,7 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B42">
         <v>4.62</v>
@@ -3011,7 +3008,7 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B43">
         <v>5.4180000000000001</v>
@@ -3025,7 +3022,7 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B44">
         <v>6</v>
@@ -3039,7 +3036,7 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B45">
         <v>6</v>
@@ -3048,7 +3045,7 @@
         <v>17.510000000000002</v>
       </c>
       <c r="D45" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E45" t="s">
         <v>18</v>
@@ -3070,7 +3067,7 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B47">
         <v>5.4180000000000001</v>
@@ -3084,7 +3081,7 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B48">
         <v>5.5369999999999999</v>
@@ -3101,7 +3098,7 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C49">
         <v>2.6974658424810825</v>
@@ -3112,7 +3109,7 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B50">
         <v>6.2869999999999999</v>
@@ -3129,7 +3126,7 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D51">
         <v>1</v>

</xml_diff>

<commit_message>
Lots of ugly code to get NEu working correctly. State functions will need to be reorganized for clarity. Also split functions into 3 files (state, national, both).
</commit_message>
<xml_diff>
--- a/data/carbon_factors.xlsx
+++ b/data/carbon_factors.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/corra_joseph_epa_gov/Documents/Profile/Documents/Fossil Fuels/Fossil Fuels/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="59" documentId="8_{272D798C-3231-4784-9687-9176A8284688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4509351-B9C7-4A45-A634-A90D0519E190}"/>
+  <xr:revisionPtr revIDLastSave="61" documentId="8_{272D798C-3231-4784-9687-9176A8284688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B19851B6-D42E-4B6B-ADF1-C0AA00A69C46}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-60" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{3ECB161D-927E-4A86-B5AC-7932B52A7390}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="factors_variable" sheetId="1" r:id="rId1"/>
     <sheet name="factors_fixed" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterate="1" iterateDelta="1.0000000000000001E-5" calcOnSave="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -84,9 +84,6 @@
     <t>Distillate Fuel Oil</t>
   </si>
   <si>
-    <t>Industrial Coking Coal</t>
-  </si>
-  <si>
     <t>Coal</t>
   </si>
   <si>
@@ -226,6 +223,9 @@
   </si>
   <si>
     <t>Other Oils</t>
+  </si>
+  <si>
+    <t>Coking Coal</t>
   </si>
 </sst>
 </file>
@@ -1120,7 +1120,7 @@
     </row>
     <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B6">
         <v>17.146363636363635</v>
@@ -2297,7 +2297,7 @@
     </row>
     <row r="17" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>15</v>
+        <v>62</v>
       </c>
       <c r="B17">
         <v>25.532291814167994</v>
@@ -2420,27 +2420,27 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E1" t="s">
         <v>53</v>
-      </c>
-      <c r="E1" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" t="s">
         <v>16</v>
-      </c>
-      <c r="B2" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -2448,10 +2448,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -2462,10 +2462,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -2473,13 +2473,13 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>62</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -2493,10 +2493,10 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -2504,10 +2504,10 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C7">
         <v>27.85</v>
@@ -2518,16 +2518,16 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" t="s">
         <v>20</v>
       </c>
-      <c r="B8" t="s">
-        <v>21</v>
-      </c>
       <c r="C8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
@@ -2535,10 +2535,10 @@
         <v>4</v>
       </c>
       <c r="B9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -2546,7 +2546,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B10">
         <v>22.3</v>
@@ -2563,7 +2563,7 @@
         <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
@@ -2571,10 +2571,10 @@
         <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -2582,7 +2582,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C13">
         <v>14.47</v>
@@ -2593,18 +2593,18 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C14">
         <v>14.47</v>
       </c>
       <c r="E14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C15">
         <v>14.92</v>
@@ -2615,15 +2615,15 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" t="s">
         <v>27</v>
-      </c>
-      <c r="B16" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B17">
         <v>6.6360000000000001</v>
@@ -2640,7 +2640,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B18">
         <v>5.048</v>
@@ -2657,10 +2657,10 @@
         <v>14</v>
       </c>
       <c r="B19" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C19" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D19">
         <v>1</v>
@@ -2677,7 +2677,7 @@
         <v>5.67</v>
       </c>
       <c r="C20" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D20">
         <v>1</v>
@@ -2685,7 +2685,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B21">
         <v>5.67</v>
@@ -2699,7 +2699,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B22">
         <v>5.67</v>
@@ -2713,13 +2713,13 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B23">
         <v>3.8410000000000002</v>
       </c>
       <c r="C23" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D23">
         <v>1</v>
@@ -2733,7 +2733,7 @@
         <v>3.867</v>
       </c>
       <c r="C24" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D24">
         <v>1</v>
@@ -2741,21 +2741,21 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B25" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C25" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E25" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B26">
         <v>6.0650000000000004</v>
@@ -2775,10 +2775,10 @@
         <v>7</v>
       </c>
       <c r="B27" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C27" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D27">
         <v>1</v>
@@ -2786,10 +2786,10 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B28" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C28">
         <v>19.22</v>
@@ -2800,7 +2800,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B29">
         <v>6.2869999999999999</v>
@@ -2817,7 +2817,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B30">
         <v>5.2480000000000002</v>
@@ -2829,17 +2829,17 @@
         <v>1</v>
       </c>
       <c r="E30" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C32">
         <v>18.87</v>
@@ -2856,7 +2856,7 @@
         <v>5.8</v>
       </c>
       <c r="C33" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D33">
         <v>1</v>
@@ -2867,7 +2867,7 @@
         <v>9</v>
       </c>
       <c r="C34" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D34">
         <v>1</v>
@@ -2881,7 +2881,7 @@
         <v>5.7960000000000003</v>
       </c>
       <c r="C35" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D35">
         <v>1</v>
@@ -2892,7 +2892,7 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B36">
         <v>5.8</v>
@@ -2909,7 +2909,7 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B37">
         <v>5.2480000000000002</v>
@@ -2921,12 +2921,12 @@
         <v>1</v>
       </c>
       <c r="E37" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B38">
         <v>5.8250000000000002</v>
@@ -2938,12 +2938,12 @@
         <v>1</v>
       </c>
       <c r="E38" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B39">
         <v>4.6379999999999999</v>
@@ -2955,15 +2955,15 @@
         <v>1</v>
       </c>
       <c r="E39" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
+        <v>40</v>
+      </c>
+      <c r="B40" t="s">
         <v>41</v>
-      </c>
-      <c r="B40" t="s">
-        <v>42</v>
       </c>
       <c r="C40">
         <v>19.37</v>
@@ -2972,12 +2972,12 @@
         <v>1</v>
       </c>
       <c r="E40" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B41">
         <v>6.024</v>
@@ -2994,7 +2994,7 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B42">
         <v>4.62</v>
@@ -3008,7 +3008,7 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B43">
         <v>5.4180000000000001</v>
@@ -3022,7 +3022,7 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B44">
         <v>6</v>
@@ -3036,7 +3036,7 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B45">
         <v>6</v>
@@ -3045,10 +3045,10 @@
         <v>17.510000000000002</v>
       </c>
       <c r="D45" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E45" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.35">
@@ -3059,7 +3059,7 @@
         <v>5.8250000000000002</v>
       </c>
       <c r="C46" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D46">
         <v>1</v>
@@ -3067,7 +3067,7 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B47">
         <v>5.4180000000000001</v>
@@ -3081,7 +3081,7 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B48">
         <v>5.5369999999999999</v>
@@ -3098,7 +3098,7 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C49">
         <v>2.6974658424810825</v>
@@ -3109,7 +3109,7 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B50">
         <v>6.2869999999999999</v>
@@ -3126,7 +3126,7 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D51">
         <v>1</v>

</xml_diff>

<commit_message>
Cleaned up NEu calculations through major restructuring--now mirrors the other sectors. haven't verified invDB output yet
</commit_message>
<xml_diff>
--- a/data/carbon_factors.xlsx
+++ b/data/carbon_factors.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/corra_joseph_epa_gov/Documents/Profile/Documents/Fossil Fuels/Fossil Fuels/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="61" documentId="8_{272D798C-3231-4784-9687-9176A8284688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B19851B6-D42E-4B6B-ADF1-C0AA00A69C46}"/>
+  <xr:revisionPtr revIDLastSave="62" documentId="8_{272D798C-3231-4784-9687-9176A8284688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{468B1936-1D3C-4367-BF7E-30841BDADA79}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-60" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{3ECB161D-927E-4A86-B5AC-7932B52A7390}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="64">
   <si>
     <t>Fuel Type</t>
   </si>
@@ -226,6 +226,9 @@
   </si>
   <si>
     <t>Coking Coal</t>
+  </si>
+  <si>
+    <t>Miscellaneous Petroleum Products</t>
   </si>
 </sst>
 </file>
@@ -2875,7 +2878,7 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>10</v>
+        <v>63</v>
       </c>
       <c r="B35">
         <v>5.7960000000000003</v>

</xml_diff>

<commit_message>
Fixed a couple of lingering problems with NEU calcs.
</commit_message>
<xml_diff>
--- a/data/carbon_factors.xlsx
+++ b/data/carbon_factors.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/corra_joseph_epa_gov/Documents/Profile/Documents/Fossil Fuels/Fossil Fuels/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="62" documentId="8_{272D798C-3231-4784-9687-9176A8284688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{468B1936-1D3C-4367-BF7E-30841BDADA79}"/>
+  <xr:revisionPtr revIDLastSave="63" documentId="8_{272D798C-3231-4784-9687-9176A8284688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7E9A3D26-CDDF-4978-BF9B-71D9B50CF8D0}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-60" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{3ECB161D-927E-4A86-B5AC-7932B52A7390}"/>
+    <workbookView xWindow="28680" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{3ECB161D-927E-4A86-B5AC-7932B52A7390}"/>
   </bookViews>
   <sheets>
     <sheet name="factors_variable" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="63">
   <si>
     <t>Fuel Type</t>
   </si>
@@ -67,9 +67,6 @@
   </si>
   <si>
     <t>MoGas Blend Components</t>
-  </si>
-  <si>
-    <t>Misc. Products</t>
   </si>
   <si>
     <t>Unfinished Oils</t>
@@ -1123,7 +1120,7 @@
     </row>
     <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B6">
         <v>17.146363636363635</v>
@@ -1765,7 +1762,7 @@
     </row>
     <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>62</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -1872,7 +1869,7 @@
     </row>
     <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B13">
         <v>20.14625771551724</v>
@@ -1979,7 +1976,7 @@
     </row>
     <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B14">
         <v>20.14625771551724</v>
@@ -2086,7 +2083,7 @@
     </row>
     <row r="15" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B15">
         <v>14.455165742468415</v>
@@ -2193,7 +2190,7 @@
     </row>
     <row r="16" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B16">
         <v>20.170000000000002</v>
@@ -2300,7 +2297,7 @@
     </row>
     <row r="17" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B17">
         <v>25.532291814167994</v>
@@ -2423,27 +2420,27 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E1" t="s">
         <v>52</v>
-      </c>
-      <c r="E1" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
         <v>15</v>
-      </c>
-      <c r="B2" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -2451,10 +2448,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -2465,10 +2462,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -2476,13 +2473,13 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -2496,10 +2493,10 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -2507,10 +2504,10 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C7">
         <v>27.85</v>
@@ -2521,16 +2518,16 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" t="s">
         <v>19</v>
       </c>
-      <c r="B8" t="s">
-        <v>20</v>
-      </c>
       <c r="C8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
@@ -2538,10 +2535,10 @@
         <v>4</v>
       </c>
       <c r="B9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -2549,7 +2546,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B10">
         <v>22.3</v>
@@ -2563,21 +2560,21 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -2585,7 +2582,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C13">
         <v>14.47</v>
@@ -2596,18 +2593,18 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C14">
         <v>14.47</v>
       </c>
       <c r="E14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C15">
         <v>14.92</v>
@@ -2618,15 +2615,15 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
+        <v>25</v>
+      </c>
+      <c r="B16" t="s">
         <v>26</v>
-      </c>
-      <c r="B16" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B17">
         <v>6.6360000000000001</v>
@@ -2643,7 +2640,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B18">
         <v>5.048</v>
@@ -2657,13 +2654,13 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B19" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C19" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D19">
         <v>1</v>
@@ -2680,7 +2677,7 @@
         <v>5.67</v>
       </c>
       <c r="C20" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D20">
         <v>1</v>
@@ -2688,7 +2685,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B21">
         <v>5.67</v>
@@ -2702,7 +2699,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B22">
         <v>5.67</v>
@@ -2716,13 +2713,13 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B23">
         <v>3.8410000000000002</v>
       </c>
       <c r="C23" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D23">
         <v>1</v>
@@ -2736,7 +2733,7 @@
         <v>3.867</v>
       </c>
       <c r="C24" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D24">
         <v>1</v>
@@ -2744,21 +2741,21 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B25" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C25" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E25" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B26">
         <v>6.0650000000000004</v>
@@ -2778,10 +2775,10 @@
         <v>7</v>
       </c>
       <c r="B27" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C27" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D27">
         <v>1</v>
@@ -2789,10 +2786,10 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B28" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C28">
         <v>19.22</v>
@@ -2803,7 +2800,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B29">
         <v>6.2869999999999999</v>
@@ -2820,7 +2817,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B30">
         <v>5.2480000000000002</v>
@@ -2832,17 +2829,17 @@
         <v>1</v>
       </c>
       <c r="E30" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C32">
         <v>18.87</v>
@@ -2853,13 +2850,13 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B33">
         <v>5.8</v>
       </c>
       <c r="C33" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D33">
         <v>1</v>
@@ -2870,7 +2867,7 @@
         <v>9</v>
       </c>
       <c r="C34" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D34">
         <v>1</v>
@@ -2878,13 +2875,13 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B35">
         <v>5.7960000000000003</v>
       </c>
       <c r="C35" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D35">
         <v>1</v>
@@ -2895,7 +2892,7 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B36">
         <v>5.8</v>
@@ -2912,7 +2909,7 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B37">
         <v>5.2480000000000002</v>
@@ -2924,12 +2921,12 @@
         <v>1</v>
       </c>
       <c r="E37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B38">
         <v>5.8250000000000002</v>
@@ -2941,12 +2938,12 @@
         <v>1</v>
       </c>
       <c r="E38" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B39">
         <v>4.6379999999999999</v>
@@ -2958,15 +2955,15 @@
         <v>1</v>
       </c>
       <c r="E39" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
+        <v>39</v>
+      </c>
+      <c r="B40" t="s">
         <v>40</v>
-      </c>
-      <c r="B40" t="s">
-        <v>41</v>
       </c>
       <c r="C40">
         <v>19.37</v>
@@ -2975,12 +2972,12 @@
         <v>1</v>
       </c>
       <c r="E40" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B41">
         <v>6.024</v>
@@ -2997,7 +2994,7 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B42">
         <v>4.62</v>
@@ -3011,7 +3008,7 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B43">
         <v>5.4180000000000001</v>
@@ -3025,7 +3022,7 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B44">
         <v>6</v>
@@ -3039,7 +3036,7 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B45">
         <v>6</v>
@@ -3048,21 +3045,21 @@
         <v>17.510000000000002</v>
       </c>
       <c r="D45" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E45" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B46">
         <v>5.8250000000000002</v>
       </c>
       <c r="C46" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D46">
         <v>1</v>
@@ -3070,7 +3067,7 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B47">
         <v>5.4180000000000001</v>
@@ -3084,7 +3081,7 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B48">
         <v>5.5369999999999999</v>
@@ -3101,7 +3098,7 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C49">
         <v>2.6974658424810825</v>
@@ -3112,7 +3109,7 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B50">
         <v>6.2869999999999999</v>
@@ -3129,7 +3126,7 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D51">
         <v>1</v>

</xml_diff>